<commit_message>
Ekg_report_daterange picker placeholder and shift time colen fixed
</commit_message>
<xml_diff>
--- a/media/downloads/Cabin_crew_inbound_trips.xlsx
+++ b/media/downloads/Cabin_crew_inbound_trips.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="174" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="32">
   <si>
     <t>DATE</t>
   </si>
@@ -46,12 +46,12 @@
     <t>06:30</t>
   </si>
   <si>
-    <t>07:30</t>
-  </si>
-  <si>
     <t>09:30</t>
   </si>
   <si>
+    <t>13:30</t>
+  </si>
+  <si>
     <t>14:30</t>
   </si>
   <si>
@@ -73,46 +73,40 @@
     <t>MILLINUM TOWER, GROSVENOUR</t>
   </si>
   <si>
+    <t>7 PEARLS</t>
+  </si>
+  <si>
+    <t>SABREEN, FALTAT, MANAZIL TOWER</t>
+  </si>
+  <si>
+    <t>GARHOUD TOWERS</t>
+  </si>
+  <si>
+    <t>TECOM 1,2</t>
+  </si>
+  <si>
     <t>DSO</t>
   </si>
   <si>
+    <t>SONBOULAH, GARHOUD TOWERS</t>
+  </si>
+  <si>
+    <t>MILLINUM TOWER, PINK, GROSVENOUR</t>
+  </si>
+  <si>
+    <t>PARK ZABEEL 1,2, 7 PEARLS</t>
+  </si>
+  <si>
     <t>EM6, QAMZI</t>
   </si>
   <si>
-    <t>SABREEN, FALTAT, MANAZIL TOWER</t>
-  </si>
-  <si>
-    <t>GARHOUD TOWERS</t>
-  </si>
-  <si>
-    <t>TECOM 1,2</t>
-  </si>
-  <si>
-    <t>7 PEARLS</t>
-  </si>
-  <si>
-    <t>SONBOULAH, GARHOUD TOWERS</t>
-  </si>
-  <si>
-    <t>MILLINUM TOWER, PINK, GROSVENOUR</t>
-  </si>
-  <si>
-    <t>PARK ZABEEL 1,2, 7 PEARLS</t>
-  </si>
-  <si>
-    <t>EM6</t>
+    <t>PINK, GROSVENOUR</t>
   </si>
   <si>
     <t>FALTAT</t>
   </si>
   <si>
-    <t>PINK, GROSVENOUR</t>
-  </si>
-  <si>
     <t>SARAB</t>
-  </si>
-  <si>
-    <t>PARK ZABEEL 1,2</t>
   </si>
   <si>
     <t>EAC-C</t>
@@ -473,7 +467,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F43"/>
+  <dimension ref="A1:F36"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
@@ -510,10 +504,10 @@
         <v>13</v>
       </c>
       <c r="E2" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="F2">
-        <v>27</v>
+        <v>14</v>
       </c>
     </row>
     <row r="3" spans="1:6">
@@ -530,10 +524,10 @@
         <v>14</v>
       </c>
       <c r="E3" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="F3">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="4" spans="1:6">
@@ -550,10 +544,10 @@
         <v>15</v>
       </c>
       <c r="E4" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="F4">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="5" spans="1:6">
@@ -570,7 +564,7 @@
         <v>16</v>
       </c>
       <c r="E5" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="F5">
         <v>5</v>
@@ -590,10 +584,10 @@
         <v>17</v>
       </c>
       <c r="E6" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="F6">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="7" spans="1:6">
@@ -610,7 +604,7 @@
         <v>18</v>
       </c>
       <c r="E7" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="F7">
         <v>6</v>
@@ -630,10 +624,10 @@
         <v>19</v>
       </c>
       <c r="E8" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="F8">
-        <v>5</v>
+        <v>9</v>
       </c>
     </row>
     <row r="9" spans="1:6">
@@ -647,13 +641,13 @@
         <v>8</v>
       </c>
       <c r="D9" t="s">
-        <v>20</v>
+        <v>13</v>
       </c>
       <c r="E9" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="F9">
-        <v>12</v>
+        <v>19</v>
       </c>
     </row>
     <row r="10" spans="1:6">
@@ -670,10 +664,10 @@
         <v>14</v>
       </c>
       <c r="E10" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="F10">
-        <v>15</v>
+        <v>27</v>
       </c>
     </row>
     <row r="11" spans="1:6">
@@ -687,13 +681,13 @@
         <v>8</v>
       </c>
       <c r="D11" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E11" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="F11">
-        <v>16</v>
+        <v>19</v>
       </c>
     </row>
     <row r="12" spans="1:6">
@@ -707,13 +701,13 @@
         <v>8</v>
       </c>
       <c r="D12" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E12" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="F12">
-        <v>11</v>
+        <v>16</v>
       </c>
     </row>
     <row r="13" spans="1:6">
@@ -727,13 +721,13 @@
         <v>8</v>
       </c>
       <c r="D13" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E13" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="F13">
-        <v>5</v>
+        <v>12</v>
       </c>
     </row>
     <row r="14" spans="1:6">
@@ -750,10 +744,10 @@
         <v>18</v>
       </c>
       <c r="E14" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="F14">
-        <v>5</v>
+        <v>10</v>
       </c>
     </row>
     <row r="15" spans="1:6">
@@ -767,10 +761,10 @@
         <v>8</v>
       </c>
       <c r="D15" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="E15" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="F15">
         <v>5</v>
@@ -787,13 +781,13 @@
         <v>8</v>
       </c>
       <c r="D16" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="E16" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="F16">
-        <v>5</v>
+        <v>10</v>
       </c>
     </row>
     <row r="17" spans="1:6">
@@ -801,7 +795,7 @@
         <v>6</v>
       </c>
       <c r="B17">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C17" t="s">
         <v>9</v>
@@ -810,10 +804,10 @@
         <v>13</v>
       </c>
       <c r="E17" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="F17">
-        <v>51</v>
+        <v>29</v>
       </c>
     </row>
     <row r="18" spans="1:6">
@@ -821,7 +815,7 @@
         <v>6</v>
       </c>
       <c r="B18">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C18" t="s">
         <v>9</v>
@@ -830,10 +824,10 @@
         <v>14</v>
       </c>
       <c r="E18" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="F18">
-        <v>35</v>
+        <v>14</v>
       </c>
     </row>
     <row r="19" spans="1:6">
@@ -847,13 +841,13 @@
         <v>9</v>
       </c>
       <c r="D19" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="E19" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="F19">
-        <v>17</v>
+        <v>19</v>
       </c>
     </row>
     <row r="20" spans="1:6">
@@ -867,13 +861,13 @@
         <v>9</v>
       </c>
       <c r="D20" t="s">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="E20" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="F20">
-        <v>26</v>
+        <v>17</v>
       </c>
     </row>
     <row r="21" spans="1:6">
@@ -887,13 +881,13 @@
         <v>9</v>
       </c>
       <c r="D21" t="s">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="E21" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="F21">
-        <v>36</v>
+        <v>48</v>
       </c>
     </row>
     <row r="22" spans="1:6">
@@ -910,10 +904,10 @@
         <v>26</v>
       </c>
       <c r="E22" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="F22">
-        <v>54</v>
+        <v>45</v>
       </c>
     </row>
     <row r="23" spans="1:6">
@@ -921,19 +915,19 @@
         <v>6</v>
       </c>
       <c r="B23">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C23" t="s">
         <v>9</v>
       </c>
       <c r="D23" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="E23" t="s">
+        <v>31</v>
+      </c>
+      <c r="F23">
         <v>33</v>
-      </c>
-      <c r="F23">
-        <v>64</v>
       </c>
     </row>
     <row r="24" spans="1:6">
@@ -941,19 +935,19 @@
         <v>6</v>
       </c>
       <c r="B24">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C24" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D24" t="s">
-        <v>19</v>
+        <v>27</v>
       </c>
       <c r="E24" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="F24">
-        <v>38</v>
+        <v>5</v>
       </c>
     </row>
     <row r="25" spans="1:6">
@@ -967,13 +961,13 @@
         <v>10</v>
       </c>
       <c r="D25" t="s">
-        <v>28</v>
+        <v>21</v>
       </c>
       <c r="E25" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="F25">
-        <v>6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="26" spans="1:6">
@@ -987,13 +981,13 @@
         <v>10</v>
       </c>
       <c r="D26" t="s">
-        <v>14</v>
+        <v>28</v>
       </c>
       <c r="E26" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="F26">
-        <v>6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="27" spans="1:6">
@@ -1007,13 +1001,13 @@
         <v>10</v>
       </c>
       <c r="D27" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="E27" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="F27">
-        <v>5</v>
+        <v>11</v>
       </c>
     </row>
     <row r="28" spans="1:6">
@@ -1024,16 +1018,16 @@
         <v>1</v>
       </c>
       <c r="C28" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D28" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="E28" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="F28">
-        <v>5</v>
+        <v>9</v>
       </c>
     </row>
     <row r="29" spans="1:6">
@@ -1044,13 +1038,13 @@
         <v>1</v>
       </c>
       <c r="C29" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D29" t="s">
-        <v>17</v>
+        <v>29</v>
       </c>
       <c r="E29" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="F29">
         <v>5</v>
@@ -1064,16 +1058,16 @@
         <v>1</v>
       </c>
       <c r="C30" t="s">
+        <v>12</v>
+      </c>
+      <c r="D30" t="s">
+        <v>27</v>
+      </c>
+      <c r="E30" t="s">
+        <v>31</v>
+      </c>
+      <c r="F30">
         <v>10</v>
-      </c>
-      <c r="D30" t="s">
-        <v>30</v>
-      </c>
-      <c r="E30" t="s">
-        <v>33</v>
-      </c>
-      <c r="F30">
-        <v>7</v>
       </c>
     </row>
     <row r="31" spans="1:6">
@@ -1084,16 +1078,16 @@
         <v>1</v>
       </c>
       <c r="C31" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D31" t="s">
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="E31" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="F31">
-        <v>9</v>
+        <v>5</v>
       </c>
     </row>
     <row r="32" spans="1:6">
@@ -1104,16 +1098,16 @@
         <v>1</v>
       </c>
       <c r="C32" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D32" t="s">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="E32" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="F32">
-        <v>8</v>
+        <v>17</v>
       </c>
     </row>
     <row r="33" spans="1:6">
@@ -1124,16 +1118,16 @@
         <v>1</v>
       </c>
       <c r="C33" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D33" t="s">
-        <v>31</v>
+        <v>21</v>
       </c>
       <c r="E33" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="F33">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="34" spans="1:6">
@@ -1144,13 +1138,13 @@
         <v>1</v>
       </c>
       <c r="C34" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D34" t="s">
         <v>22</v>
       </c>
       <c r="E34" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="F34">
         <v>5</v>
@@ -1164,16 +1158,16 @@
         <v>1</v>
       </c>
       <c r="C35" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D35" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="E35" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="F35">
-        <v>5</v>
+        <v>26</v>
       </c>
     </row>
     <row r="36" spans="1:6">
@@ -1184,156 +1178,16 @@
         <v>1</v>
       </c>
       <c r="C36" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D36" t="s">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="E36" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="F36">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="37" spans="1:6">
-      <c r="A37" t="s">
-        <v>6</v>
-      </c>
-      <c r="B37">
-        <v>1</v>
-      </c>
-      <c r="C37" t="s">
-        <v>11</v>
-      </c>
-      <c r="D37" t="s">
-        <v>32</v>
-      </c>
-      <c r="E37" t="s">
-        <v>33</v>
-      </c>
-      <c r="F37">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="38" spans="1:6">
-      <c r="A38" t="s">
-        <v>6</v>
-      </c>
-      <c r="B38">
-        <v>1</v>
-      </c>
-      <c r="C38" t="s">
-        <v>12</v>
-      </c>
-      <c r="D38" t="s">
-        <v>31</v>
-      </c>
-      <c r="E38" t="s">
-        <v>33</v>
-      </c>
-      <c r="F38">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="39" spans="1:6">
-      <c r="A39" t="s">
-        <v>6</v>
-      </c>
-      <c r="B39">
-        <v>1</v>
-      </c>
-      <c r="C39" t="s">
-        <v>12</v>
-      </c>
-      <c r="D39" t="s">
-        <v>29</v>
-      </c>
-      <c r="E39" t="s">
-        <v>33</v>
-      </c>
-      <c r="F39">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="40" spans="1:6">
-      <c r="A40" t="s">
-        <v>6</v>
-      </c>
-      <c r="B40">
-        <v>1</v>
-      </c>
-      <c r="C40" t="s">
-        <v>12</v>
-      </c>
-      <c r="D40" t="s">
-        <v>23</v>
-      </c>
-      <c r="E40" t="s">
-        <v>33</v>
-      </c>
-      <c r="F40">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="41" spans="1:6">
-      <c r="A41" t="s">
-        <v>6</v>
-      </c>
-      <c r="B41">
-        <v>1</v>
-      </c>
-      <c r="C41" t="s">
-        <v>12</v>
-      </c>
-      <c r="D41" t="s">
-        <v>18</v>
-      </c>
-      <c r="E41" t="s">
-        <v>33</v>
-      </c>
-      <c r="F41">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="42" spans="1:6">
-      <c r="A42" t="s">
-        <v>6</v>
-      </c>
-      <c r="B42">
-        <v>3</v>
-      </c>
-      <c r="C42" t="s">
-        <v>12</v>
-      </c>
-      <c r="D42" t="s">
-        <v>27</v>
-      </c>
-      <c r="E42" t="s">
-        <v>33</v>
-      </c>
-      <c r="F42">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="43" spans="1:6">
-      <c r="A43" t="s">
-        <v>6</v>
-      </c>
-      <c r="B43">
-        <v>1</v>
-      </c>
-      <c r="C43" t="s">
-        <v>12</v>
-      </c>
-      <c r="D43" t="s">
-        <v>19</v>
-      </c>
-      <c r="E43" t="s">
-        <v>33</v>
-      </c>
-      <c r="F43">
-        <v>10</v>
+        <v>5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Cabincrew outbound Combining Non-Empty Columns & Skipping Empty Cells
</commit_message>
<xml_diff>
--- a/media/downloads/Cabin_crew_inbound_trips.xlsx
+++ b/media/downloads/Cabin_crew_inbound_trips.xlsx
@@ -34,7 +34,7 @@
     <t>CREW</t>
   </si>
   <si>
-    <t>13-Jan</t>
+    <t>19-Jan</t>
   </si>
   <si>
     <t>05:00</t>
@@ -55,27 +55,30 @@
     <t>14:30</t>
   </si>
   <si>
+    <t>EM6, QAMZI</t>
+  </si>
+  <si>
+    <t>SARAB, SAFA</t>
+  </si>
+  <si>
+    <t>SABREEN, FALTAT</t>
+  </si>
+  <si>
+    <t>SONBOULAH</t>
+  </si>
+  <si>
+    <t>TECOM 1,2, DR.KHALIFA</t>
+  </si>
+  <si>
+    <t>MILLINUM TOWER, GROSVENOUR</t>
+  </si>
+  <si>
+    <t>7 PEARLS</t>
+  </si>
+  <si>
     <t>EM6, TALAL, QAMZI</t>
   </si>
   <si>
-    <t>SARAB, SAFA</t>
-  </si>
-  <si>
-    <t>SABREEN, FALTAT</t>
-  </si>
-  <si>
-    <t>SONBOULAH</t>
-  </si>
-  <si>
-    <t>TECOM 1,2, DR.KHALIFA</t>
-  </si>
-  <si>
-    <t>MILLINUM TOWER, GROSVENOUR</t>
-  </si>
-  <si>
-    <t>7 PEARLS</t>
-  </si>
-  <si>
     <t>SABREEN, FALTAT, MANAZIL TOWER</t>
   </si>
   <si>
@@ -95,9 +98,6 @@
   </si>
   <si>
     <t>PARK ZABEEL 1,2, 7 PEARLS</t>
-  </si>
-  <si>
-    <t>EM6, QAMZI</t>
   </si>
   <si>
     <t>PINK, GROSVENOUR</t>
@@ -507,7 +507,7 @@
         <v>31</v>
       </c>
       <c r="F2">
-        <v>14</v>
+        <v>8</v>
       </c>
     </row>
     <row r="3" spans="1:6">
@@ -641,7 +641,7 @@
         <v>8</v>
       </c>
       <c r="D9" t="s">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="E9" t="s">
         <v>31</v>
@@ -681,7 +681,7 @@
         <v>8</v>
       </c>
       <c r="D11" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E11" t="s">
         <v>31</v>
@@ -701,7 +701,7 @@
         <v>8</v>
       </c>
       <c r="D12" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E12" t="s">
         <v>31</v>
@@ -721,7 +721,7 @@
         <v>8</v>
       </c>
       <c r="D13" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E13" t="s">
         <v>31</v>
@@ -781,7 +781,7 @@
         <v>8</v>
       </c>
       <c r="D16" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E16" t="s">
         <v>31</v>
@@ -801,7 +801,7 @@
         <v>9</v>
       </c>
       <c r="D17" t="s">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="E17" t="s">
         <v>31</v>
@@ -841,7 +841,7 @@
         <v>9</v>
       </c>
       <c r="D19" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E19" t="s">
         <v>31</v>
@@ -881,7 +881,7 @@
         <v>9</v>
       </c>
       <c r="D21" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E21" t="s">
         <v>31</v>
@@ -901,7 +901,7 @@
         <v>9</v>
       </c>
       <c r="D22" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E22" t="s">
         <v>31</v>
@@ -921,7 +921,7 @@
         <v>9</v>
       </c>
       <c r="D23" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E23" t="s">
         <v>31</v>
@@ -941,7 +941,7 @@
         <v>10</v>
       </c>
       <c r="D24" t="s">
-        <v>27</v>
+        <v>13</v>
       </c>
       <c r="E24" t="s">
         <v>31</v>
@@ -961,7 +961,7 @@
         <v>10</v>
       </c>
       <c r="D25" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E25" t="s">
         <v>31</v>
@@ -1001,7 +1001,7 @@
         <v>10</v>
       </c>
       <c r="D27" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E27" t="s">
         <v>31</v>
@@ -1021,7 +1021,7 @@
         <v>11</v>
       </c>
       <c r="D28" t="s">
-        <v>27</v>
+        <v>13</v>
       </c>
       <c r="E28" t="s">
         <v>31</v>
@@ -1061,7 +1061,7 @@
         <v>12</v>
       </c>
       <c r="D30" t="s">
-        <v>27</v>
+        <v>13</v>
       </c>
       <c r="E30" t="s">
         <v>31</v>
@@ -1101,7 +1101,7 @@
         <v>12</v>
       </c>
       <c r="D32" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E32" t="s">
         <v>31</v>
@@ -1121,7 +1121,7 @@
         <v>12</v>
       </c>
       <c r="D33" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E33" t="s">
         <v>31</v>
@@ -1141,7 +1141,7 @@
         <v>12</v>
       </c>
       <c r="D34" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E34" t="s">
         <v>31</v>
@@ -1161,7 +1161,7 @@
         <v>12</v>
       </c>
       <c r="D35" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E35" t="s">
         <v>31</v>
@@ -1181,7 +1181,7 @@
         <v>12</v>
       </c>
       <c r="D36" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E36" t="s">
         <v>31</v>

</xml_diff>

<commit_message>
admin.py for bus master table and user ui page add new column error fixed
</commit_message>
<xml_diff>
--- a/media/downloads/Cabin_crew_inbound_trips.xlsx
+++ b/media/downloads/Cabin_crew_inbound_trips.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="206" uniqueCount="38">
   <si>
     <t>DATE</t>
   </si>
@@ -34,7 +34,7 @@
     <t>CREW</t>
   </si>
   <si>
-    <t>19-Jan</t>
+    <t>28-Feb</t>
   </si>
   <si>
     <t>05:00</t>
@@ -46,67 +46,85 @@
     <t>06:30</t>
   </si>
   <si>
+    <t>07:30</t>
+  </si>
+  <si>
     <t>09:30</t>
   </si>
   <si>
-    <t>13:30</t>
-  </si>
-  <si>
-    <t>14:30</t>
-  </si>
-  <si>
-    <t>EM6, QAMZI</t>
+    <t>13:00</t>
+  </si>
+  <si>
+    <t>14:00</t>
+  </si>
+  <si>
+    <t>15:00</t>
+  </si>
+  <si>
+    <t>EM6</t>
+  </si>
+  <si>
+    <t>SARAB</t>
+  </si>
+  <si>
+    <t>TECOM 1,2</t>
+  </si>
+  <si>
+    <t>GROSVENOUR</t>
+  </si>
+  <si>
+    <t>EM6, TALAL, QAMZI</t>
+  </si>
+  <si>
+    <t>FALTAT, MANAZIL TOWER</t>
+  </si>
+  <si>
+    <t>GARHOUD TOWERS</t>
+  </si>
+  <si>
+    <t>7 PEARLS</t>
+  </si>
+  <si>
+    <t>DSO</t>
   </si>
   <si>
     <t>SARAB, SAFA</t>
   </si>
   <si>
-    <t>SABREEN, FALTAT</t>
-  </si>
-  <si>
-    <t>SONBOULAH</t>
+    <t>SABREEN, FALTAT, MANAZIL TOWER</t>
+  </si>
+  <si>
+    <t>SONBOULAH, GARHOUD TOWERS</t>
   </si>
   <si>
     <t>TECOM 1,2, DR.KHALIFA</t>
   </si>
   <si>
+    <t>MILLINUM TOWER, PINK, GROSVENOUR</t>
+  </si>
+  <si>
+    <t>PARK ZABEEL 1,2, 7 PEARLS</t>
+  </si>
+  <si>
+    <t>EM6, TALAL</t>
+  </si>
+  <si>
+    <t>FALTAT</t>
+  </si>
+  <si>
+    <t>PARK ZABEEL 1,2</t>
+  </si>
+  <si>
     <t>MILLINUM TOWER, GROSVENOUR</t>
   </si>
   <si>
-    <t>7 PEARLS</t>
-  </si>
-  <si>
-    <t>EM6, TALAL, QAMZI</t>
-  </si>
-  <si>
-    <t>SABREEN, FALTAT, MANAZIL TOWER</t>
-  </si>
-  <si>
-    <t>GARHOUD TOWERS</t>
-  </si>
-  <si>
-    <t>TECOM 1,2</t>
-  </si>
-  <si>
-    <t>DSO</t>
-  </si>
-  <si>
-    <t>SONBOULAH, GARHOUD TOWERS</t>
-  </si>
-  <si>
-    <t>MILLINUM TOWER, PINK, GROSVENOUR</t>
-  </si>
-  <si>
-    <t>PARK ZABEEL 1,2, 7 PEARLS</t>
-  </si>
-  <si>
-    <t>PINK, GROSVENOUR</t>
-  </si>
-  <si>
-    <t>FALTAT</t>
-  </si>
-  <si>
-    <t>SARAB</t>
+    <t>TALAL, QAMZI</t>
+  </si>
+  <si>
+    <t>SABREEN, MANAZIL TOWER</t>
+  </si>
+  <si>
+    <t>MILLINUM TOWER</t>
   </si>
   <si>
     <t>EAC-C</t>
@@ -467,7 +485,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F36"/>
+  <dimension ref="A1:F51"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
@@ -501,13 +519,13 @@
         <v>7</v>
       </c>
       <c r="D2" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="E2" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="F2">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="3" spans="1:6">
@@ -521,13 +539,13 @@
         <v>7</v>
       </c>
       <c r="D3" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="E3" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="F3">
-        <v>10</v>
+        <v>5</v>
       </c>
     </row>
     <row r="4" spans="1:6">
@@ -541,13 +559,13 @@
         <v>7</v>
       </c>
       <c r="D4" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="E4" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="F4">
-        <v>5</v>
+        <v>16</v>
       </c>
     </row>
     <row r="5" spans="1:6">
@@ -561,13 +579,13 @@
         <v>7</v>
       </c>
       <c r="D5" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="E5" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="F5">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="6" spans="1:6">
@@ -578,16 +596,16 @@
         <v>1</v>
       </c>
       <c r="C6" t="s">
+        <v>8</v>
+      </c>
+      <c r="D6" t="s">
+        <v>19</v>
+      </c>
+      <c r="E6" t="s">
+        <v>37</v>
+      </c>
+      <c r="F6">
         <v>7</v>
-      </c>
-      <c r="D6" t="s">
-        <v>17</v>
-      </c>
-      <c r="E6" t="s">
-        <v>31</v>
-      </c>
-      <c r="F6">
-        <v>5</v>
       </c>
     </row>
     <row r="7" spans="1:6">
@@ -598,16 +616,16 @@
         <v>1</v>
       </c>
       <c r="C7" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D7" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="E7" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="F7">
-        <v>6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="8" spans="1:6">
@@ -618,16 +636,16 @@
         <v>1</v>
       </c>
       <c r="C8" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D8" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="E8" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="F8">
-        <v>9</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9" spans="1:6">
@@ -641,13 +659,13 @@
         <v>8</v>
       </c>
       <c r="D9" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="E9" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="F9">
-        <v>19</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10" spans="1:6">
@@ -661,13 +679,13 @@
         <v>8</v>
       </c>
       <c r="D10" t="s">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="E10" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="F10">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="11" spans="1:6">
@@ -681,13 +699,13 @@
         <v>8</v>
       </c>
       <c r="D11" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="E11" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="F11">
-        <v>19</v>
+        <v>30</v>
       </c>
     </row>
     <row r="12" spans="1:6">
@@ -695,19 +713,19 @@
         <v>6</v>
       </c>
       <c r="B12">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C12" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D12" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="E12" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="F12">
-        <v>16</v>
+        <v>64</v>
       </c>
     </row>
     <row r="13" spans="1:6">
@@ -715,19 +733,19 @@
         <v>6</v>
       </c>
       <c r="B13">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C13" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D13" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E13" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="F13">
-        <v>12</v>
+        <v>52</v>
       </c>
     </row>
     <row r="14" spans="1:6">
@@ -735,19 +753,19 @@
         <v>6</v>
       </c>
       <c r="B14">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C14" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D14" t="s">
-        <v>18</v>
+        <v>25</v>
       </c>
       <c r="E14" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="F14">
-        <v>10</v>
+        <v>43</v>
       </c>
     </row>
     <row r="15" spans="1:6">
@@ -755,19 +773,19 @@
         <v>6</v>
       </c>
       <c r="B15">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C15" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D15" t="s">
-        <v>19</v>
+        <v>26</v>
       </c>
       <c r="E15" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="F15">
-        <v>5</v>
+        <v>37</v>
       </c>
     </row>
     <row r="16" spans="1:6">
@@ -778,16 +796,16 @@
         <v>1</v>
       </c>
       <c r="C16" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D16" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="E16" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="F16">
-        <v>10</v>
+        <v>21</v>
       </c>
     </row>
     <row r="17" spans="1:6">
@@ -801,13 +819,13 @@
         <v>9</v>
       </c>
       <c r="D17" t="s">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="E17" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="F17">
-        <v>29</v>
+        <v>25</v>
       </c>
     </row>
     <row r="18" spans="1:6">
@@ -821,13 +839,13 @@
         <v>9</v>
       </c>
       <c r="D18" t="s">
-        <v>14</v>
+        <v>29</v>
       </c>
       <c r="E18" t="s">
+        <v>37</v>
+      </c>
+      <c r="F18">
         <v>31</v>
-      </c>
-      <c r="F18">
-        <v>14</v>
       </c>
     </row>
     <row r="19" spans="1:6">
@@ -835,19 +853,19 @@
         <v>6</v>
       </c>
       <c r="B19">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C19" t="s">
         <v>9</v>
       </c>
       <c r="D19" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="E19" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="F19">
-        <v>19</v>
+        <v>39</v>
       </c>
     </row>
     <row r="20" spans="1:6">
@@ -858,16 +876,16 @@
         <v>1</v>
       </c>
       <c r="C20" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D20" t="s">
-        <v>17</v>
+        <v>30</v>
       </c>
       <c r="E20" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="F20">
-        <v>17</v>
+        <v>5</v>
       </c>
     </row>
     <row r="21" spans="1:6">
@@ -875,19 +893,19 @@
         <v>6</v>
       </c>
       <c r="B21">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C21" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D21" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="E21" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="F21">
-        <v>48</v>
+        <v>5</v>
       </c>
     </row>
     <row r="22" spans="1:6">
@@ -895,19 +913,19 @@
         <v>6</v>
       </c>
       <c r="B22">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C22" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D22" t="s">
-        <v>27</v>
+        <v>18</v>
       </c>
       <c r="E22" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="F22">
-        <v>45</v>
+        <v>5</v>
       </c>
     </row>
     <row r="23" spans="1:6">
@@ -915,19 +933,19 @@
         <v>6</v>
       </c>
       <c r="B23">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C23" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D23" t="s">
-        <v>24</v>
+        <v>32</v>
       </c>
       <c r="E23" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="F23">
-        <v>33</v>
+        <v>5</v>
       </c>
     </row>
     <row r="24" spans="1:6">
@@ -941,13 +959,13 @@
         <v>10</v>
       </c>
       <c r="D24" t="s">
-        <v>13</v>
+        <v>23</v>
       </c>
       <c r="E24" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="F24">
-        <v>5</v>
+        <v>16</v>
       </c>
     </row>
     <row r="25" spans="1:6">
@@ -958,16 +976,16 @@
         <v>1</v>
       </c>
       <c r="C25" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D25" t="s">
-        <v>22</v>
+        <v>30</v>
       </c>
       <c r="E25" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="F25">
-        <v>2</v>
+        <v>11</v>
       </c>
     </row>
     <row r="26" spans="1:6">
@@ -978,16 +996,16 @@
         <v>1</v>
       </c>
       <c r="C26" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D26" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="E26" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="F26">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="27" spans="1:6">
@@ -998,16 +1016,16 @@
         <v>1</v>
       </c>
       <c r="C27" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D27" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="E27" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="F27">
-        <v>11</v>
+        <v>9</v>
       </c>
     </row>
     <row r="28" spans="1:6">
@@ -1021,13 +1039,13 @@
         <v>11</v>
       </c>
       <c r="D28" t="s">
-        <v>13</v>
+        <v>27</v>
       </c>
       <c r="E28" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="F28">
-        <v>9</v>
+        <v>2</v>
       </c>
     </row>
     <row r="29" spans="1:6">
@@ -1041,13 +1059,13 @@
         <v>11</v>
       </c>
       <c r="D29" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="E29" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="F29">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="30" spans="1:6">
@@ -1058,13 +1076,13 @@
         <v>1</v>
       </c>
       <c r="C30" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D30" t="s">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="E30" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="F30">
         <v>10</v>
@@ -1078,16 +1096,16 @@
         <v>1</v>
       </c>
       <c r="C31" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D31" t="s">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="E31" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="F31">
-        <v>5</v>
+        <v>22</v>
       </c>
     </row>
     <row r="32" spans="1:6">
@@ -1101,13 +1119,13 @@
         <v>12</v>
       </c>
       <c r="D32" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="E32" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="F32">
-        <v>17</v>
+        <v>14</v>
       </c>
     </row>
     <row r="33" spans="1:6">
@@ -1121,13 +1139,13 @@
         <v>12</v>
       </c>
       <c r="D33" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="E33" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="F33">
-        <v>5</v>
+        <v>12</v>
       </c>
     </row>
     <row r="34" spans="1:6">
@@ -1141,10 +1159,10 @@
         <v>12</v>
       </c>
       <c r="D34" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="E34" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="F34">
         <v>5</v>
@@ -1161,13 +1179,13 @@
         <v>12</v>
       </c>
       <c r="D35" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E35" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="F35">
-        <v>26</v>
+        <v>10</v>
       </c>
     </row>
     <row r="36" spans="1:6">
@@ -1181,12 +1199,312 @@
         <v>12</v>
       </c>
       <c r="D36" t="s">
+        <v>33</v>
+      </c>
+      <c r="E36" t="s">
+        <v>37</v>
+      </c>
+      <c r="F36">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6">
+      <c r="A37" t="s">
+        <v>6</v>
+      </c>
+      <c r="B37">
+        <v>1</v>
+      </c>
+      <c r="C37" t="s">
+        <v>12</v>
+      </c>
+      <c r="D37" t="s">
+        <v>29</v>
+      </c>
+      <c r="E37" t="s">
+        <v>37</v>
+      </c>
+      <c r="F37">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6">
+      <c r="A38" t="s">
+        <v>6</v>
+      </c>
+      <c r="B38">
+        <v>1</v>
+      </c>
+      <c r="C38" t="s">
+        <v>13</v>
+      </c>
+      <c r="D38" t="s">
+        <v>30</v>
+      </c>
+      <c r="E38" t="s">
+        <v>37</v>
+      </c>
+      <c r="F38">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6">
+      <c r="A39" t="s">
+        <v>6</v>
+      </c>
+      <c r="B39">
+        <v>2</v>
+      </c>
+      <c r="C39" t="s">
+        <v>13</v>
+      </c>
+      <c r="D39" t="s">
         <v>24</v>
       </c>
-      <c r="E36" t="s">
-        <v>31</v>
-      </c>
-      <c r="F36">
+      <c r="E39" t="s">
+        <v>37</v>
+      </c>
+      <c r="F39">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6">
+      <c r="A40" t="s">
+        <v>6</v>
+      </c>
+      <c r="B40">
+        <v>1</v>
+      </c>
+      <c r="C40" t="s">
+        <v>13</v>
+      </c>
+      <c r="D40" t="s">
+        <v>25</v>
+      </c>
+      <c r="E40" t="s">
+        <v>37</v>
+      </c>
+      <c r="F40">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6">
+      <c r="A41" t="s">
+        <v>6</v>
+      </c>
+      <c r="B41">
+        <v>1</v>
+      </c>
+      <c r="C41" t="s">
+        <v>13</v>
+      </c>
+      <c r="D41" t="s">
+        <v>21</v>
+      </c>
+      <c r="E41" t="s">
+        <v>37</v>
+      </c>
+      <c r="F41">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6">
+      <c r="A42" t="s">
+        <v>6</v>
+      </c>
+      <c r="B42">
+        <v>2</v>
+      </c>
+      <c r="C42" t="s">
+        <v>13</v>
+      </c>
+      <c r="D42" t="s">
+        <v>27</v>
+      </c>
+      <c r="E42" t="s">
+        <v>37</v>
+      </c>
+      <c r="F42">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6">
+      <c r="A43" t="s">
+        <v>6</v>
+      </c>
+      <c r="B43">
+        <v>1</v>
+      </c>
+      <c r="C43" t="s">
+        <v>13</v>
+      </c>
+      <c r="D43" t="s">
+        <v>28</v>
+      </c>
+      <c r="E43" t="s">
+        <v>37</v>
+      </c>
+      <c r="F43">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6">
+      <c r="A44" t="s">
+        <v>6</v>
+      </c>
+      <c r="B44">
+        <v>1</v>
+      </c>
+      <c r="C44" t="s">
+        <v>13</v>
+      </c>
+      <c r="D44" t="s">
+        <v>29</v>
+      </c>
+      <c r="E44" t="s">
+        <v>37</v>
+      </c>
+      <c r="F44">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6">
+      <c r="A45" t="s">
+        <v>6</v>
+      </c>
+      <c r="B45">
+        <v>1</v>
+      </c>
+      <c r="C45" t="s">
+        <v>14</v>
+      </c>
+      <c r="D45" t="s">
+        <v>34</v>
+      </c>
+      <c r="E45" t="s">
+        <v>37</v>
+      </c>
+      <c r="F45">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6">
+      <c r="A46" t="s">
+        <v>6</v>
+      </c>
+      <c r="B46">
+        <v>1</v>
+      </c>
+      <c r="C46" t="s">
+        <v>14</v>
+      </c>
+      <c r="D46" t="s">
+        <v>24</v>
+      </c>
+      <c r="E46" t="s">
+        <v>37</v>
+      </c>
+      <c r="F46">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6">
+      <c r="A47" t="s">
+        <v>6</v>
+      </c>
+      <c r="B47">
+        <v>1</v>
+      </c>
+      <c r="C47" t="s">
+        <v>14</v>
+      </c>
+      <c r="D47" t="s">
+        <v>35</v>
+      </c>
+      <c r="E47" t="s">
+        <v>37</v>
+      </c>
+      <c r="F47">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6">
+      <c r="A48" t="s">
+        <v>6</v>
+      </c>
+      <c r="B48">
+        <v>1</v>
+      </c>
+      <c r="C48" t="s">
+        <v>14</v>
+      </c>
+      <c r="D48" t="s">
+        <v>21</v>
+      </c>
+      <c r="E48" t="s">
+        <v>37</v>
+      </c>
+      <c r="F48">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6">
+      <c r="A49" t="s">
+        <v>6</v>
+      </c>
+      <c r="B49">
+        <v>1</v>
+      </c>
+      <c r="C49" t="s">
+        <v>14</v>
+      </c>
+      <c r="D49" t="s">
+        <v>27</v>
+      </c>
+      <c r="E49" t="s">
+        <v>37</v>
+      </c>
+      <c r="F49">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6">
+      <c r="A50" t="s">
+        <v>6</v>
+      </c>
+      <c r="B50">
+        <v>1</v>
+      </c>
+      <c r="C50" t="s">
+        <v>14</v>
+      </c>
+      <c r="D50" t="s">
+        <v>36</v>
+      </c>
+      <c r="E50" t="s">
+        <v>37</v>
+      </c>
+      <c r="F50">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6">
+      <c r="A51" t="s">
+        <v>6</v>
+      </c>
+      <c r="B51">
+        <v>1</v>
+      </c>
+      <c r="C51" t="s">
+        <v>14</v>
+      </c>
+      <c r="D51" t="s">
+        <v>32</v>
+      </c>
+      <c r="E51" t="s">
+        <v>37</v>
+      </c>
+      <c r="F51">
         <v>5</v>
       </c>
     </row>

</xml_diff>